<commit_message>
feat(support): resolve live email delivery, smtp sender alignment, and admin email audit logs
</commit_message>
<xml_diff>
--- a/docs/VNPay_Sandbox_Test_Cards_Full.xlsx
+++ b/docs/VNPay_Sandbox_Test_Cards_Full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lunara\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB5FB96-7AAC-4BA4-855D-20995E02AAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F07640-D561-46B2-A24C-5328E805C7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="The test VNPay" sheetId="1" r:id="rId1"/>
@@ -423,6 +423,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -430,9 +433,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,55 +709,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
     </row>
     <row r="3" spans="1:13" ht="22.35" customHeight="1">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
     </row>
     <row r="5" spans="1:13" ht="24" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -968,7 +968,7 @@
         <v>44</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="8" t="s">
         <v>45</v>
       </c>
       <c r="J11" s="2" t="s">

</xml_diff>